<commit_message>
error en la vista uploadDrive con las importaciones de los models
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
+++ b/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
@@ -808,14 +808,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="n">
-        <v>45180.47732763336</v>
+        <v>45237</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -853,20 +849,6 @@
       </c>
       <c r="E10" s="6" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25" ht="18" customHeight="1" s="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
@@ -898,7 +880,7 @@
       </c>
       <c r="C26" s="26" t="n"/>
       <c r="D26" s="27" t="n">
-        <v>160.866</v>
+        <v>175.344</v>
       </c>
       <c r="E26" s="28" t="n"/>
       <c r="F26" s="28" t="n"/>
@@ -916,7 +898,7 @@
       </c>
       <c r="C27" s="26" t="n"/>
       <c r="D27" s="27" t="n">
-        <v>203.305</v>
+        <v>221.602</v>
       </c>
       <c r="E27" s="28" t="n"/>
       <c r="F27" s="28" t="n"/>
@@ -934,7 +916,7 @@
       </c>
       <c r="C28" s="24" t="n"/>
       <c r="D28" s="27" t="n">
-        <v>247.861</v>
+        <v>300</v>
       </c>
       <c r="E28" s="28" t="n"/>
       <c r="F28" s="28" t="n"/>
@@ -942,8 +924,6 @@
     <row r="29">
       <c r="E29" s="28" t="n"/>
     </row>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32" ht="19.5" customHeight="1" s="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
@@ -951,15 +931,12 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="8" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="9" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -969,13 +946,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
mas error al subir al drive super extraño
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
+++ b/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
@@ -808,7 +808,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="n">
-        <v>45237</v>
+        <v>45238</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -946,13 +946,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A9:D9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
funcionalidad upload drive sin fallos y mejore la vista step2
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
+++ b/LISTAS/ma/BISAGRAS ESCALERA DISMAY.xlsx
@@ -946,13 +946,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="A9:D9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>